<commit_message>
Fix to add snack and meal cost goals.
</commit_message>
<xml_diff>
--- a/InterestCalculation.xlsx
+++ b/InterestCalculation.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Take Home Calc 43" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Inheritance Calculator 1000000" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -416,91 +416,1080 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Take Home Calculator</t>
+          <t>Inheritance Calculation</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Base pay: $43.00</t>
+          <t>Initial Inheritance: $1000000.00</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>Details</t>
+          <t>Planned Usage</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Potential Amounts</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Personal Spend</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Amount Invested</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pay frequency: hourly</t>
+          <t>Estate Tax: 10.00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Adjusted Base Pay</t>
+          <t>Total Inherited</t>
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>1720</v>
+        <v>450000</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>400000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Goal pay frequency: weekly</t>
+          <t>Percent Inherited: 50.00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tax Reduction</t>
+          <t>Debt to pay off</t>
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>206.4</v>
+        <v>50000</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>395500</v>
       </c>
     </row>
     <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Debt: $50000.00</t>
+        </is>
+      </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Set Aside for 401K/IRA</t>
+          <t>Personal Usage</t>
         </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>172</v>
+        <v>112500</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>9000</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>391000</v>
       </c>
     </row>
     <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Desired Personal Spend: 25.00</t>
+        </is>
+      </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Total Reductions</t>
+          <t>Remainder</t>
         </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>378.4</v>
+        <v>287500</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>13500</v>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>386500</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Amount Remaining</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="n">
-        <v>1341.6</v>
+      <c r="D7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>382000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>22500</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>377500</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="D9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>27000</v>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>373000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="D10" t="n">
+        <v>7</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>31500</v>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>368500</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="D11" t="n">
+        <v>8</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>36000</v>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>364000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="D12" t="n">
+        <v>9</v>
+      </c>
+      <c r="E12" s="1" t="n">
+        <v>40500</v>
+      </c>
+      <c r="F12" s="1" t="n">
+        <v>359500</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="D13" t="n">
+        <v>10</v>
+      </c>
+      <c r="E13" s="1" t="n">
+        <v>45000</v>
+      </c>
+      <c r="F13" s="1" t="n">
+        <v>355000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="D14" t="n">
+        <v>11</v>
+      </c>
+      <c r="E14" s="1" t="n">
+        <v>49500</v>
+      </c>
+      <c r="F14" s="1" t="n">
+        <v>350500</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="D15" t="n">
+        <v>12</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>54000</v>
+      </c>
+      <c r="F15" s="1" t="n">
+        <v>346000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="D16" t="n">
+        <v>13</v>
+      </c>
+      <c r="E16" s="1" t="n">
+        <v>58500</v>
+      </c>
+      <c r="F16" s="1" t="n">
+        <v>341500</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="D17" t="n">
+        <v>14</v>
+      </c>
+      <c r="E17" s="1" t="n">
+        <v>63000.00000000001</v>
+      </c>
+      <c r="F17" s="1" t="n">
+        <v>337000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="D18" t="n">
+        <v>15</v>
+      </c>
+      <c r="E18" s="1" t="n">
+        <v>67500</v>
+      </c>
+      <c r="F18" s="1" t="n">
+        <v>332500</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="D19" t="n">
+        <v>16</v>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>72000</v>
+      </c>
+      <c r="F19" s="1" t="n">
+        <v>328000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="D20" t="n">
+        <v>17</v>
+      </c>
+      <c r="E20" s="1" t="n">
+        <v>76500</v>
+      </c>
+      <c r="F20" s="1" t="n">
+        <v>323500</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="D21" t="n">
+        <v>18</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>81000</v>
+      </c>
+      <c r="F21" s="1" t="n">
+        <v>319000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="D22" t="n">
+        <v>19</v>
+      </c>
+      <c r="E22" s="1" t="n">
+        <v>85500</v>
+      </c>
+      <c r="F22" s="1" t="n">
+        <v>314500</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="D23" t="n">
+        <v>20</v>
+      </c>
+      <c r="E23" s="1" t="n">
+        <v>90000</v>
+      </c>
+      <c r="F23" s="1" t="n">
+        <v>310000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="D24" t="n">
+        <v>21</v>
+      </c>
+      <c r="E24" s="1" t="n">
+        <v>94500</v>
+      </c>
+      <c r="F24" s="1" t="n">
+        <v>305500</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="D25" t="n">
+        <v>22</v>
+      </c>
+      <c r="E25" s="1" t="n">
+        <v>99000</v>
+      </c>
+      <c r="F25" s="1" t="n">
+        <v>301000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="D26" t="n">
+        <v>23</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>103500</v>
+      </c>
+      <c r="F26" s="1" t="n">
+        <v>296500</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="D27" t="n">
+        <v>24</v>
+      </c>
+      <c r="E27" s="1" t="n">
+        <v>108000</v>
+      </c>
+      <c r="F27" s="1" t="n">
+        <v>292000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="D28" t="n">
+        <v>25</v>
+      </c>
+      <c r="E28" s="1" t="n">
+        <v>112500</v>
+      </c>
+      <c r="F28" s="1" t="n">
+        <v>287500</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="D29" t="n">
+        <v>26</v>
+      </c>
+      <c r="E29" s="1" t="n">
+        <v>117000</v>
+      </c>
+      <c r="F29" s="1" t="n">
+        <v>283000</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="D30" t="n">
+        <v>27</v>
+      </c>
+      <c r="E30" s="1" t="n">
+        <v>121500</v>
+      </c>
+      <c r="F30" s="1" t="n">
+        <v>278500</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="D31" t="n">
+        <v>28</v>
+      </c>
+      <c r="E31" s="1" t="n">
+        <v>126000</v>
+      </c>
+      <c r="F31" s="1" t="n">
+        <v>274000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="D32" t="n">
+        <v>29</v>
+      </c>
+      <c r="E32" s="1" t="n">
+        <v>130500</v>
+      </c>
+      <c r="F32" s="1" t="n">
+        <v>269500</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="D33" t="n">
+        <v>30</v>
+      </c>
+      <c r="E33" s="1" t="n">
+        <v>135000</v>
+      </c>
+      <c r="F33" s="1" t="n">
+        <v>265000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="D34" t="n">
+        <v>31</v>
+      </c>
+      <c r="E34" s="1" t="n">
+        <v>139500</v>
+      </c>
+      <c r="F34" s="1" t="n">
+        <v>260500</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="D35" t="n">
+        <v>32</v>
+      </c>
+      <c r="E35" s="1" t="n">
+        <v>144000</v>
+      </c>
+      <c r="F35" s="1" t="n">
+        <v>256000</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="D36" t="n">
+        <v>33</v>
+      </c>
+      <c r="E36" s="1" t="n">
+        <v>148500</v>
+      </c>
+      <c r="F36" s="1" t="n">
+        <v>251500</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="D37" t="n">
+        <v>34</v>
+      </c>
+      <c r="E37" s="1" t="n">
+        <v>153000</v>
+      </c>
+      <c r="F37" s="1" t="n">
+        <v>247000</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="D38" t="n">
+        <v>35</v>
+      </c>
+      <c r="E38" s="1" t="n">
+        <v>157500</v>
+      </c>
+      <c r="F38" s="1" t="n">
+        <v>242500</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="D39" t="n">
+        <v>36</v>
+      </c>
+      <c r="E39" s="1" t="n">
+        <v>162000</v>
+      </c>
+      <c r="F39" s="1" t="n">
+        <v>238000</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="D40" t="n">
+        <v>37</v>
+      </c>
+      <c r="E40" s="1" t="n">
+        <v>166500</v>
+      </c>
+      <c r="F40" s="1" t="n">
+        <v>233500</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="D41" t="n">
+        <v>38</v>
+      </c>
+      <c r="E41" s="1" t="n">
+        <v>171000</v>
+      </c>
+      <c r="F41" s="1" t="n">
+        <v>229000</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="D42" t="n">
+        <v>39</v>
+      </c>
+      <c r="E42" s="1" t="n">
+        <v>175500</v>
+      </c>
+      <c r="F42" s="1" t="n">
+        <v>224500</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="D43" t="n">
+        <v>40</v>
+      </c>
+      <c r="E43" s="1" t="n">
+        <v>180000</v>
+      </c>
+      <c r="F43" s="1" t="n">
+        <v>220000</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="D44" t="n">
+        <v>41</v>
+      </c>
+      <c r="E44" s="1" t="n">
+        <v>184500</v>
+      </c>
+      <c r="F44" s="1" t="n">
+        <v>215500</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="D45" t="n">
+        <v>42</v>
+      </c>
+      <c r="E45" s="1" t="n">
+        <v>189000</v>
+      </c>
+      <c r="F45" s="1" t="n">
+        <v>211000</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="D46" t="n">
+        <v>43</v>
+      </c>
+      <c r="E46" s="1" t="n">
+        <v>193500</v>
+      </c>
+      <c r="F46" s="1" t="n">
+        <v>206500</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="D47" t="n">
+        <v>44</v>
+      </c>
+      <c r="E47" s="1" t="n">
+        <v>198000</v>
+      </c>
+      <c r="F47" s="1" t="n">
+        <v>202000</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="D48" t="n">
+        <v>45</v>
+      </c>
+      <c r="E48" s="1" t="n">
+        <v>202500</v>
+      </c>
+      <c r="F48" s="1" t="n">
+        <v>197500</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="D49" t="n">
+        <v>46</v>
+      </c>
+      <c r="E49" s="1" t="n">
+        <v>207000</v>
+      </c>
+      <c r="F49" s="1" t="n">
+        <v>193000</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="D50" t="n">
+        <v>47</v>
+      </c>
+      <c r="E50" s="1" t="n">
+        <v>211500</v>
+      </c>
+      <c r="F50" s="1" t="n">
+        <v>188500</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="D51" t="n">
+        <v>48</v>
+      </c>
+      <c r="E51" s="1" t="n">
+        <v>216000</v>
+      </c>
+      <c r="F51" s="1" t="n">
+        <v>184000</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="D52" t="n">
+        <v>49</v>
+      </c>
+      <c r="E52" s="1" t="n">
+        <v>220500</v>
+      </c>
+      <c r="F52" s="1" t="n">
+        <v>179500</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="D53" t="n">
+        <v>50</v>
+      </c>
+      <c r="E53" s="1" t="n">
+        <v>225000</v>
+      </c>
+      <c r="F53" s="1" t="n">
+        <v>175000</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="D54" t="n">
+        <v>51</v>
+      </c>
+      <c r="E54" s="1" t="n">
+        <v>229500</v>
+      </c>
+      <c r="F54" s="1" t="n">
+        <v>170500</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="D55" t="n">
+        <v>52</v>
+      </c>
+      <c r="E55" s="1" t="n">
+        <v>234000</v>
+      </c>
+      <c r="F55" s="1" t="n">
+        <v>166000</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="D56" t="n">
+        <v>53</v>
+      </c>
+      <c r="E56" s="1" t="n">
+        <v>238500</v>
+      </c>
+      <c r="F56" s="1" t="n">
+        <v>161500</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="D57" t="n">
+        <v>54</v>
+      </c>
+      <c r="E57" s="1" t="n">
+        <v>243000</v>
+      </c>
+      <c r="F57" s="1" t="n">
+        <v>157000</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="D58" t="n">
+        <v>55</v>
+      </c>
+      <c r="E58" s="1" t="n">
+        <v>247500</v>
+      </c>
+      <c r="F58" s="1" t="n">
+        <v>152500</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="D59" t="n">
+        <v>56</v>
+      </c>
+      <c r="E59" s="1" t="n">
+        <v>252000</v>
+      </c>
+      <c r="F59" s="1" t="n">
+        <v>148000</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="D60" t="n">
+        <v>57</v>
+      </c>
+      <c r="E60" s="1" t="n">
+        <v>256500</v>
+      </c>
+      <c r="F60" s="1" t="n">
+        <v>143500</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="D61" t="n">
+        <v>58</v>
+      </c>
+      <c r="E61" s="1" t="n">
+        <v>261000</v>
+      </c>
+      <c r="F61" s="1" t="n">
+        <v>139000</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="D62" t="n">
+        <v>59</v>
+      </c>
+      <c r="E62" s="1" t="n">
+        <v>265500</v>
+      </c>
+      <c r="F62" s="1" t="n">
+        <v>134500</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="D63" t="n">
+        <v>60</v>
+      </c>
+      <c r="E63" s="1" t="n">
+        <v>270000</v>
+      </c>
+      <c r="F63" s="1" t="n">
+        <v>130000</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="D64" t="n">
+        <v>61</v>
+      </c>
+      <c r="E64" s="1" t="n">
+        <v>274500</v>
+      </c>
+      <c r="F64" s="1" t="n">
+        <v>125500</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="D65" t="n">
+        <v>62</v>
+      </c>
+      <c r="E65" s="1" t="n">
+        <v>279000</v>
+      </c>
+      <c r="F65" s="1" t="n">
+        <v>121000</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="D66" t="n">
+        <v>63</v>
+      </c>
+      <c r="E66" s="1" t="n">
+        <v>283500</v>
+      </c>
+      <c r="F66" s="1" t="n">
+        <v>116500</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="D67" t="n">
+        <v>64</v>
+      </c>
+      <c r="E67" s="1" t="n">
+        <v>288000</v>
+      </c>
+      <c r="F67" s="1" t="n">
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="D68" t="n">
+        <v>65</v>
+      </c>
+      <c r="E68" s="1" t="n">
+        <v>292500</v>
+      </c>
+      <c r="F68" s="1" t="n">
+        <v>107500</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="D69" t="n">
+        <v>66</v>
+      </c>
+      <c r="E69" s="1" t="n">
+        <v>297000</v>
+      </c>
+      <c r="F69" s="1" t="n">
+        <v>103000</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="D70" t="n">
+        <v>67</v>
+      </c>
+      <c r="E70" s="1" t="n">
+        <v>301500</v>
+      </c>
+      <c r="F70" s="1" t="n">
+        <v>98500</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="D71" t="n">
+        <v>68</v>
+      </c>
+      <c r="E71" s="1" t="n">
+        <v>306000</v>
+      </c>
+      <c r="F71" s="1" t="n">
+        <v>94000</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="D72" t="n">
+        <v>69</v>
+      </c>
+      <c r="E72" s="1" t="n">
+        <v>310500</v>
+      </c>
+      <c r="F72" s="1" t="n">
+        <v>89500</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="D73" t="n">
+        <v>70</v>
+      </c>
+      <c r="E73" s="1" t="n">
+        <v>315000</v>
+      </c>
+      <c r="F73" s="1" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="D74" t="n">
+        <v>71</v>
+      </c>
+      <c r="E74" s="1" t="n">
+        <v>319500</v>
+      </c>
+      <c r="F74" s="1" t="n">
+        <v>80500</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="D75" t="n">
+        <v>72</v>
+      </c>
+      <c r="E75" s="1" t="n">
+        <v>324000</v>
+      </c>
+      <c r="F75" s="1" t="n">
+        <v>76000</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="D76" t="n">
+        <v>73</v>
+      </c>
+      <c r="E76" s="1" t="n">
+        <v>328500</v>
+      </c>
+      <c r="F76" s="1" t="n">
+        <v>71500</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="D77" t="n">
+        <v>74</v>
+      </c>
+      <c r="E77" s="1" t="n">
+        <v>333000</v>
+      </c>
+      <c r="F77" s="1" t="n">
+        <v>67000</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="D78" t="n">
+        <v>75</v>
+      </c>
+      <c r="E78" s="1" t="n">
+        <v>337500</v>
+      </c>
+      <c r="F78" s="1" t="n">
+        <v>62500</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="D79" t="n">
+        <v>76</v>
+      </c>
+      <c r="E79" s="1" t="n">
+        <v>342000</v>
+      </c>
+      <c r="F79" s="1" t="n">
+        <v>58000</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="D80" t="n">
+        <v>77</v>
+      </c>
+      <c r="E80" s="1" t="n">
+        <v>346500</v>
+      </c>
+      <c r="F80" s="1" t="n">
+        <v>53500</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="D81" t="n">
+        <v>78</v>
+      </c>
+      <c r="E81" s="1" t="n">
+        <v>351000</v>
+      </c>
+      <c r="F81" s="1" t="n">
+        <v>49000</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="D82" t="n">
+        <v>79</v>
+      </c>
+      <c r="E82" s="1" t="n">
+        <v>355500</v>
+      </c>
+      <c r="F82" s="1" t="n">
+        <v>44500</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="D83" t="n">
+        <v>80</v>
+      </c>
+      <c r="E83" s="1" t="n">
+        <v>360000</v>
+      </c>
+      <c r="F83" s="1" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="D84" t="n">
+        <v>81</v>
+      </c>
+      <c r="E84" s="1" t="n">
+        <v>364500</v>
+      </c>
+      <c r="F84" s="1" t="n">
+        <v>35500</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="D85" t="n">
+        <v>82</v>
+      </c>
+      <c r="E85" s="1" t="n">
+        <v>369000</v>
+      </c>
+      <c r="F85" s="1" t="n">
+        <v>31000</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="D86" t="n">
+        <v>83</v>
+      </c>
+      <c r="E86" s="1" t="n">
+        <v>373500</v>
+      </c>
+      <c r="F86" s="1" t="n">
+        <v>26500</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="D87" t="n">
+        <v>84</v>
+      </c>
+      <c r="E87" s="1" t="n">
+        <v>378000</v>
+      </c>
+      <c r="F87" s="1" t="n">
+        <v>22000</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="D88" t="n">
+        <v>85</v>
+      </c>
+      <c r="E88" s="1" t="n">
+        <v>382500</v>
+      </c>
+      <c r="F88" s="1" t="n">
+        <v>17500</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="D89" t="n">
+        <v>86</v>
+      </c>
+      <c r="E89" s="1" t="n">
+        <v>387000</v>
+      </c>
+      <c r="F89" s="1" t="n">
+        <v>13000</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="D90" t="n">
+        <v>87</v>
+      </c>
+      <c r="E90" s="1" t="n">
+        <v>391500</v>
+      </c>
+      <c r="F90" s="1" t="n">
+        <v>8500</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="D91" t="n">
+        <v>88</v>
+      </c>
+      <c r="E91" s="1" t="n">
+        <v>396000</v>
+      </c>
+      <c r="F91" s="1" t="n">
+        <v>4000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>